<commit_message>
Add Type in Excel import
</commit_message>
<xml_diff>
--- a/public/templates/Book-Import-Template.xlsx
+++ b/public/templates/Book-Import-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\bookhub\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3A8832-E828-43C9-AF94-9A3952C148AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27C01D2-AF4F-466B-A36D-C4FBE2524724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{9DD50B20-475A-4F9F-9449-86A427C58EF4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Book Condition</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>Image</t>
+  </si>
+  <si>
+    <t>Type</t>
   </si>
 </sst>
 </file>
@@ -467,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D018F96-49E5-43E9-A10D-55C1779A262D}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -478,12 +481,12 @@
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
     <col min="8" max="8" width="20.140625" customWidth="1"/>
     <col min="9" max="9" width="43.28515625" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" customWidth="1"/>
-    <col min="12" max="12" width="19.140625" customWidth="1"/>
+    <col min="10" max="11" width="18.140625" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" customWidth="1"/>
+    <col min="13" max="13" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -515,9 +518,12 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add class and type in excel import
</commit_message>
<xml_diff>
--- a/public/templates/Book-Import-Template.xlsx
+++ b/public/templates/Book-Import-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\bookhub\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27C01D2-AF4F-466B-A36D-C4FBE2524724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D85EDAA-520D-4788-A98B-5822B02BD57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{9DD50B20-475A-4F9F-9449-86A427C58EF4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Book Condition</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <t>Class</t>
   </si>
 </sst>
 </file>
@@ -470,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D018F96-49E5-43E9-A10D-55C1779A262D}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -478,15 +481,15 @@
     <col min="3" max="4" width="34.85546875" customWidth="1"/>
     <col min="5" max="5" width="19.5703125" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
-    <col min="8" max="8" width="20.140625" customWidth="1"/>
-    <col min="9" max="9" width="43.28515625" customWidth="1"/>
-    <col min="10" max="11" width="18.140625" customWidth="1"/>
-    <col min="12" max="12" width="16.7109375" customWidth="1"/>
-    <col min="13" max="13" width="19.140625" customWidth="1"/>
+    <col min="7" max="8" width="26.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" customWidth="1"/>
+    <col min="10" max="10" width="43.28515625" customWidth="1"/>
+    <col min="11" max="12" width="18.140625" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" customWidth="1"/>
+    <col min="14" max="14" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="1" customFormat="1" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -509,21 +512,24 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>